<commit_message>
add generated expected results
</commit_message>
<xml_diff>
--- a/testcases-llm-review4-runner-ready-results.xlsx
+++ b/testcases-llm-review4-runner-ready-results.xlsx
@@ -77,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -92,6 +92,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -171,8 +174,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TestCases" displayName="TestCases" ref="A5:L156" headerRowCount="1">
-  <autoFilter ref="A5:L156"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TestCases" displayName="TestCases" ref="A5:M156" headerRowCount="1">
+  <autoFilter ref="A5:M156"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Module"/>
     <tableColumn id="2" name="Sub-module (Test Summary)"/>
@@ -480,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L156"/>
+  <dimension ref="A1:M156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -495,6 +498,7 @@
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="48" customWidth="1" min="11" max="11"/>
     <col width="56" customWidth="1" min="12" max="12"/>
+    <col width="64" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
@@ -612,6 +616,11 @@
       <c r="L5" s="4" t="inlineStr">
         <is>
           <t>Technical Evidence</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>Generated Expected Result</t>
         </is>
       </c>
     </row>
@@ -763,6 +772,11 @@
 POST | 200 | demowebshop.tricentis.com/checkout/OpcConfirmOrder/</t>
         </is>
       </c>
+      <c r="M6" s="6" t="inlineStr">
+        <is>
+          <t>The user is logged out and the demo web shop home page at demowebshop.tricentis.com/ is displayed with the Log in link visible in the header.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="72" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
@@ -830,6 +844,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/blue-jeans to demowebshop.tricentis.com/blue-jeans</t>
         </is>
       </c>
+      <c r="M7" s="6" t="inlineStr">
+        <is>
+          <t>The textbox displays the entered text 'test'.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="72" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
@@ -898,6 +917,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/blue-jeans to demowebshop.tricentis.com/blue-jeans</t>
         </is>
       </c>
+      <c r="M8" s="6" t="inlineStr">
+        <is>
+          <t>The second matching textbox displays the entered text 'test' and the first textbox still shows 'test'.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="72" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
@@ -967,6 +991,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/blue-jeans to demowebshop.tricentis.com/blue-jeans</t>
         </is>
       </c>
+      <c r="M9" s="6" t="inlineStr">
+        <is>
+          <t>The Qty: textbox displays 1 and the previously entered text values remain displayed.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="72" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
@@ -1037,6 +1066,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/blue-jeans to demowebshop.tricentis.com/</t>
         </is>
       </c>
+      <c r="M10" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to the home page at demowebshop.tricentis.com/ and the home page is displayed.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="72" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
@@ -1106,6 +1140,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to Not recorded</t>
         </is>
       </c>
+      <c r="M11" s="6" t="inlineStr">
+        <is>
+          <t>The home page at demowebshop.tricentis.com/ is displayed listing the product categories.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="72" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
@@ -1175,6 +1214,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to Not recorded</t>
         </is>
       </c>
+      <c r="M12" s="6" t="inlineStr">
+        <is>
+          <t>The product reviews for the linked product are displayed.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="72" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
@@ -1244,6 +1288,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to Not recorded</t>
         </is>
       </c>
+      <c r="M13" s="6" t="inlineStr">
+        <is>
+          <t>The add product review form is displayed for the linked product.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="72" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
@@ -1313,6 +1362,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to Not recorded</t>
         </is>
       </c>
+      <c r="M14" s="6" t="inlineStr">
+        <is>
+          <t>The Email a friend form opens for the product.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="72" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
@@ -1382,6 +1436,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to Not recorded</t>
         </is>
       </c>
+      <c r="M15" s="6" t="inlineStr">
+        <is>
+          <t>The product is added to the compare list and a confirmation notification is displayed.</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="72" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
@@ -1451,6 +1510,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to Not recorded</t>
         </is>
       </c>
+      <c r="M16" s="6" t="inlineStr">
+        <is>
+          <t>The product details page for Blue and green Sneaker is displayed.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="72" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
@@ -1520,6 +1584,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to Not recorded</t>
         </is>
       </c>
+      <c r="M17" s="6" t="inlineStr">
+        <is>
+          <t>The product details page for Blue and green Sneaker is displayed.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="72" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
@@ -1589,6 +1658,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to Not recorded</t>
         </is>
       </c>
+      <c r="M18" s="6" t="inlineStr">
+        <is>
+          <t>The product details page for Computing and Internet is displayed.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="72" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
@@ -1658,6 +1732,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to Not recorded</t>
         </is>
       </c>
+      <c r="M19" s="6" t="inlineStr">
+        <is>
+          <t>The product details page for Computing and Internet is displayed.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="72" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
@@ -1725,6 +1804,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/register</t>
         </is>
       </c>
+      <c r="M20" s="6" t="inlineStr">
+        <is>
+          <t>The registration page at demowebshop.tricentis.com/register is displayed.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="72" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
@@ -1792,6 +1876,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/login</t>
         </is>
       </c>
+      <c r="M21" s="6" t="inlineStr">
+        <is>
+          <t>The login page at demowebshop.tricentis.com/login is displayed.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="72" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
@@ -1861,6 +1950,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/cart</t>
         </is>
       </c>
+      <c r="M22" s="6" t="inlineStr">
+        <is>
+          <t>The shopping cart page at demowebshop.tricentis.com/cart is displayed showing no items.</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="72" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
@@ -1928,6 +2022,11 @@
           <t>POST | 201 | https://demowebshop.tricentis.com/addproducttocart/catalog/2/1/1</t>
         </is>
       </c>
+      <c r="M23" s="6" t="inlineStr">
+        <is>
+          <t>The item is added to the shopping cart and the cart count in the header increases.</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="72" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
@@ -1995,6 +2094,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/producttag/3/cool</t>
         </is>
       </c>
+      <c r="M24" s="6" t="inlineStr">
+        <is>
+          <t>The product listing for the 'cool' product tag is displayed at demowebshop.tricentis.com/producttag/3/cool.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="72" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
@@ -2062,6 +2166,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/apparel-shoes</t>
         </is>
       </c>
+      <c r="M25" s="6" t="inlineStr">
+        <is>
+          <t>The apparel product listing at demowebshop.tricentis.com/apparel-shoes is displayed.</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="72" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
@@ -2129,6 +2238,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/producttag/14/jeans</t>
         </is>
       </c>
+      <c r="M26" s="6" t="inlineStr">
+        <is>
+          <t>The products tagged 'jeans' are displayed at demowebshop.tricentis.com/producttag/14/jeans.</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="72" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
@@ -2196,6 +2310,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/141-inch-laptop</t>
         </is>
       </c>
+      <c r="M27" s="6" t="inlineStr">
+        <is>
+          <t>The product details page for the 14.1-inch Laptop is displayed at demowebshop.tricentis.com/141-inch-laptop.</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="72" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
@@ -2263,6 +2382,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/141-inch-laptop</t>
         </is>
       </c>
+      <c r="M28" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to demowebshop.tricentis.com/141-inch-laptop and the 14.1-inch Laptop product listing page is displayed.</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="72" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
@@ -2330,6 +2454,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/</t>
         </is>
       </c>
+      <c r="M29" s="6" t="inlineStr">
+        <is>
+          <t>The Tricentis link is activated and the user remains on the demo web shop home page at demowebshop.tricentis.com/ with the home page content displayed.</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="72" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
@@ -2397,6 +2526,11 @@
           <t>POST | 201 | https://demowebshop.tricentis.com/subscribenewsletter</t>
         </is>
       </c>
+      <c r="M30" s="6" t="inlineStr">
+        <is>
+          <t>The newsletter subscription request is submitted successfully and a confirmation message for the subscription is displayed on the page.</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="72" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
@@ -2466,6 +2600,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/wishlist</t>
         </is>
       </c>
+      <c r="M31" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to demowebshop.tricentis.com/wishlist and the wishlist page is displayed showing the wishlist items or an empty wishlist.</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="72" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
@@ -2533,6 +2672,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/</t>
         </is>
       </c>
+      <c r="M32" s="6" t="inlineStr">
+        <is>
+          <t>The keyword search is executed and the search results page lists products matching the entered term; if the term is under 3 characters, a warning message is displayed.</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="72" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
@@ -2600,6 +2744,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/books</t>
         </is>
       </c>
+      <c r="M33" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to demowebshop.tricentis.com/books and the Books category page is displayed with its product listing.</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="72" customHeight="1">
       <c r="A34" s="5" t="inlineStr">
@@ -2667,6 +2816,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/computers</t>
         </is>
       </c>
+      <c r="M34" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to demowebshop.tricentis.com/computers and the Computers category page is displayed showing its sub-categories such as Desktops, Notebooks and Accessories.</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="72" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
@@ -2734,6 +2888,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/electronics</t>
         </is>
       </c>
+      <c r="M35" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to demowebshop.tricentis.com/electronics and the Electronics category page is displayed with its product listing.</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="72" customHeight="1">
       <c r="A36" s="5" t="inlineStr">
@@ -2801,6 +2960,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/apparel-shoes</t>
         </is>
       </c>
+      <c r="M36" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to demowebshop.tricentis.com/apparel-shoes and the Apparel &amp; Shoes category page is displayed with its product listing.</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="72" customHeight="1">
       <c r="A37" s="5" t="inlineStr">
@@ -2868,6 +3032,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/digital-downloads</t>
         </is>
       </c>
+      <c r="M37" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to demowebshop.tricentis.com/digital-downloads and the Digital Downloads category page is displayed with its product listing.</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="72" customHeight="1">
       <c r="A38" s="5" t="inlineStr">
@@ -2935,6 +3104,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/jewelry</t>
         </is>
       </c>
+      <c r="M38" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to demowebshop.tricentis.com/jewelry and the Jewelry category page is displayed with its product listing.</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="72" customHeight="1">
       <c r="A39" s="5" t="inlineStr">
@@ -3002,6 +3176,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/gift-cards</t>
         </is>
       </c>
+      <c r="M39" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to demowebshop.tricentis.com/gift-cards and the Gift Cards category page is displayed with its product listing.</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="72" customHeight="1">
       <c r="A40" s="5" t="inlineStr">
@@ -3069,6 +3248,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/sitemap</t>
         </is>
       </c>
+      <c r="M40" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to demowebshop.tricentis.com/sitemap and the sitemap page is displayed listing the site categories and pages.</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="72" customHeight="1">
       <c r="A41" s="5" t="inlineStr">
@@ -3136,6 +3320,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/shipping-returns</t>
         </is>
       </c>
+      <c r="M41" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to demowebshop.tricentis.com/shipping-returns and the Shipping &amp; Returns information page is displayed.</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="72" customHeight="1">
       <c r="A42" s="5" t="inlineStr">
@@ -3203,6 +3392,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/privacy-policy</t>
         </is>
       </c>
+      <c r="M42" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to demowebshop.tricentis.com/privacy-policy and the Privacy Notice page is displayed.</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="72" customHeight="1">
       <c r="A43" s="5" t="inlineStr">
@@ -3270,6 +3464,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/conditions-of-use</t>
         </is>
       </c>
+      <c r="M43" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to demowebshop.tricentis.com/conditions-of-use and the Conditions of Use page is displayed.</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="72" customHeight="1">
       <c r="A44" s="5" t="inlineStr">
@@ -3337,6 +3536,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/about-us</t>
         </is>
       </c>
+      <c r="M44" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to demowebshop.tricentis.com/about-us and the About us page is displayed.</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="72" customHeight="1">
       <c r="A45" s="5" t="inlineStr">
@@ -3404,6 +3608,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/contactus</t>
         </is>
       </c>
+      <c r="M45" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to demowebshop.tricentis.com/contactus and the Contact us page with its contact form is displayed.</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="72" customHeight="1">
       <c r="A46" s="5" t="inlineStr">
@@ -3471,6 +3680,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/search</t>
         </is>
       </c>
+      <c r="M46" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to demowebshop.tricentis.com/search and the search page is displayed with the search form and any matching results.</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="72" customHeight="1">
       <c r="A47" s="5" t="inlineStr">
@@ -3538,6 +3752,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/news</t>
         </is>
       </c>
+      <c r="M47" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to demowebshop.tricentis.com/news and the News page is displayed listing news items.</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="72" customHeight="1">
       <c r="A48" s="5" t="inlineStr">
@@ -3605,6 +3824,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/blog</t>
         </is>
       </c>
+      <c r="M48" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to demowebshop.tricentis.com/blog and the Blog page is displayed listing blog posts.</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="72" customHeight="1">
       <c r="A49" s="5" t="inlineStr">
@@ -3672,6 +3896,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/recentlyviewedproducts</t>
         </is>
       </c>
+      <c r="M49" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to demowebshop.tricentis.com/recentlyviewedproducts and the Recently Viewed Products page is displayed listing the products recently viewed by the user.</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="72" customHeight="1">
       <c r="A50" s="5" t="inlineStr">
@@ -3739,6 +3968,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/compareproducts</t>
         </is>
       </c>
+      <c r="M50" s="6" t="inlineStr">
+        <is>
+          <t>The Compare products page opens at demowebshop.tricentis.com/compareproducts and displays the compare products list.</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="72" customHeight="1">
       <c r="A51" s="5" t="inlineStr">
@@ -3806,6 +4040,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/newproducts</t>
         </is>
       </c>
+      <c r="M51" s="6" t="inlineStr">
+        <is>
+          <t>The New products page opens at demowebshop.tricentis.com/newproducts and lists the newly added products.</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="72" customHeight="1">
       <c r="A52" s="5" t="inlineStr">
@@ -3873,6 +4112,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/customer/info</t>
         </is>
       </c>
+      <c r="M52" s="6" t="inlineStr">
+        <is>
+          <t>The My account page opens at demowebshop.tricentis.com/customer/info and displays the customer's account information form.</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="72" customHeight="1">
       <c r="A53" s="5" t="inlineStr">
@@ -3940,6 +4184,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/customer/orders</t>
         </is>
       </c>
+      <c r="M53" s="6" t="inlineStr">
+        <is>
+          <t>The Orders page opens at demowebshop.tricentis.com/customer/orders and displays the customer's order history.</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="72" customHeight="1">
       <c r="A54" s="5" t="inlineStr">
@@ -4007,6 +4256,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/customer/addresses</t>
         </is>
       </c>
+      <c r="M54" s="6" t="inlineStr">
+        <is>
+          <t>The Addresses page opens at demowebshop.tricentis.com/customer/addresses and displays the customer's saved address book.</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="72" customHeight="1">
       <c r="A55" s="5" t="inlineStr">
@@ -4074,6 +4328,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/cart</t>
         </is>
       </c>
+      <c r="M55" s="6" t="inlineStr">
+        <is>
+          <t>The Shopping cart page opens at demowebshop.tricentis.com/cart and displays the current cart contents.</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="72" customHeight="1">
       <c r="A56" s="5" t="inlineStr">
@@ -4141,6 +4400,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/wishlist</t>
         </is>
       </c>
+      <c r="M56" s="6" t="inlineStr">
+        <is>
+          <t>The Wishlist page opens at demowebshop.tricentis.com/wishlist and displays the wishlist items.</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="72" customHeight="1">
       <c r="A57" s="5" t="inlineStr">
@@ -4204,6 +4468,11 @@
       <c r="L57" s="5" t="inlineStr">
         <is>
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/news/rss/1</t>
+        </is>
+      </c>
+      <c r="M57" s="6" t="inlineStr">
+        <is>
+          <t>The RSS feed opens at demowebshop.tricentis.com/news/rss/1 and displays the news feed content.</t>
         </is>
       </c>
     </row>
@@ -4269,6 +4538,11 @@
       <c r="L58" s="5" t="inlineStr">
         <is>
           <t>Page | status not applicable | demowebshop.tricentis.com/ to Not recorded</t>
+        </is>
+      </c>
+      <c r="M58" s="6" t="inlineStr">
+        <is>
+          <t>The nopCommerce link navigates from the starting page to the nopCommerce website.</t>
         </is>
       </c>
     </row>
@@ -4337,6 +4611,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/</t>
         </is>
       </c>
+      <c r="M59" s="6" t="inlineStr">
+        <is>
+          <t>The Facebook link opens in a new tab or window and the demo web shop home page at demowebshop.tricentis.com/ remains displayed.</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="72" customHeight="1">
       <c r="A60" s="5" t="inlineStr">
@@ -4403,6 +4682,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/</t>
         </is>
       </c>
+      <c r="M60" s="6" t="inlineStr">
+        <is>
+          <t>The Twitter link opens in a new tab or window and the demo web shop home page at demowebshop.tricentis.com/ remains displayed.</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="72" customHeight="1">
       <c r="A61" s="5" t="inlineStr">
@@ -4469,6 +4753,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/</t>
         </is>
       </c>
+      <c r="M61" s="6" t="inlineStr">
+        <is>
+          <t>The YouTube link opens in a new tab or window and the demo web shop home page at demowebshop.tricentis.com/ remains displayed.</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="72" customHeight="1">
       <c r="A62" s="5" t="inlineStr">
@@ -4535,6 +4824,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/</t>
         </is>
       </c>
+      <c r="M62" s="6" t="inlineStr">
+        <is>
+          <t>The Google+ link opens in a new tab or window and the demo web shop home page at demowebshop.tricentis.com/ remains displayed.</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="72" customHeight="1">
       <c r="A63" s="5" t="inlineStr">
@@ -4602,6 +4896,11 @@
           <t>POST | 201 | https://demowebshop.tricentis.com/addproducttocart/catalog/31/1/1</t>
         </is>
       </c>
+      <c r="M63" s="6" t="inlineStr">
+        <is>
+          <t>The product is added to the shopping cart and a confirmation message or updated cart count is displayed.</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="72" customHeight="1">
       <c r="A64" s="5" t="inlineStr">
@@ -4666,6 +4965,11 @@
           <t>POST | 201 | https://demowebshop.tricentis.com/addproducttocart/catalog/72/1/1</t>
         </is>
       </c>
+      <c r="M64" s="6" t="inlineStr">
+        <is>
+          <t>The product is added to the shopping cart and a confirmation message or updated cart count is displayed.</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="72" customHeight="1">
       <c r="A65" s="5" t="inlineStr">
@@ -4728,6 +5032,11 @@
       <c r="L65" s="5" t="inlineStr">
         <is>
           <t>POST | 201 | https://demowebshop.tricentis.com/addproducttocart/catalog/16/1/1</t>
+        </is>
+      </c>
+      <c r="M65" s="6" t="inlineStr">
+        <is>
+          <t>The product is added to the shopping cart and a confirmation message or updated cart count is displayed.</t>
         </is>
       </c>
     </row>
@@ -4797,6 +5106,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to demowebshop.tricentis.com/apparel-shoes</t>
         </is>
       </c>
+      <c r="M66" s="6" t="inlineStr">
+        <is>
+          <t>The Apparel &amp; Shoes category page opens at demowebshop.tricentis.com/apparel-shoes and lists products in that category.</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="72" customHeight="1">
       <c r="A67" s="5" t="inlineStr">
@@ -4865,6 +5179,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/newproducts to demowebshop.tricentis.com/phone-cover</t>
         </is>
       </c>
+      <c r="M67" s="6" t="inlineStr">
+        <is>
+          <t>The Phone Cover product details page opens at demowebshop.tricentis.com/phone-cover and shows the product name, image, and price.</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="72" customHeight="1">
       <c r="A68" s="5" t="inlineStr">
@@ -4933,6 +5252,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/newproducts to demowebshop.tricentis.com/phone-cover</t>
         </is>
       </c>
+      <c r="M68" s="6" t="inlineStr">
+        <is>
+          <t>The Phone Cover product details page opens at demowebshop.tricentis.com/phone-cover and shows the product name, image, and price.</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="72" customHeight="1">
       <c r="A69" s="5" t="inlineStr">
@@ -5001,6 +5325,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/newproducts to demowebshop.tricentis.com/tblue-jeans</t>
         </is>
       </c>
+      <c r="M69" s="6" t="inlineStr">
+        <is>
+          <t>The TBlue Jeans product details page opens at demowebshop.tricentis.com/tblue-jeans and shows the product name, image, and price.</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="72" customHeight="1">
       <c r="A70" s="5" t="inlineStr">
@@ -5069,6 +5398,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/newproducts to demowebshop.tricentis.com/tblue-jeans</t>
         </is>
       </c>
+      <c r="M70" s="6" t="inlineStr">
+        <is>
+          <t>The TBlue Jeans product details page opens at demowebshop.tricentis.com/tblue-jeans and shows the product name, image, and price.</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="72" customHeight="1">
       <c r="A71" s="5" t="inlineStr">
@@ -5137,6 +5471,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/newproducts to demowebshop.tricentis.com/copy-of-computing-and-internet</t>
         </is>
       </c>
+      <c r="M71" s="6" t="inlineStr">
+        <is>
+          <t>The product details page opens at demowebshop.tricentis.com/copy-of-computing-and-internet and shows the product name, image, and price.</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="72" customHeight="1">
       <c r="A72" s="5" t="inlineStr">
@@ -5205,6 +5544,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/newproducts to demowebshop.tricentis.com/copy-of-computing-and-internet</t>
         </is>
       </c>
+      <c r="M72" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to the Copy of Computing and Internet EX product details page, showing its product name and price.</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="72" customHeight="1">
       <c r="A73" s="5" t="inlineStr">
@@ -5273,6 +5617,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/newproducts to demowebshop.tricentis.com/fiction-ex</t>
         </is>
       </c>
+      <c r="M73" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to the Picture of Fiction EX product details page, showing the product name and price.</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="72" customHeight="1">
       <c r="A74" s="5" t="inlineStr">
@@ -5341,6 +5690,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/newproducts to demowebshop.tricentis.com/fiction-ex</t>
         </is>
       </c>
+      <c r="M74" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to the Fiction EX product details page, showing the product name and price.</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="72" customHeight="1">
       <c r="A75" s="5" t="inlineStr">
@@ -5409,6 +5763,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/newproducts to demowebshop.tricentis.com/create-it-yourself-jewelry</t>
         </is>
       </c>
+      <c r="M75" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to the Picture of Create Your Own Jewelry product details page, showing the product name and price.</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="72" customHeight="1">
       <c r="A76" s="5" t="inlineStr">
@@ -5477,6 +5836,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/newproducts to demowebshop.tricentis.com/create-it-yourself-jewelry</t>
         </is>
       </c>
+      <c r="M76" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to the Create Your Own Jewelry product details page, showing the product name and price.</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="72" customHeight="1">
       <c r="A77" s="5" t="inlineStr">
@@ -5545,6 +5909,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/newproducts to demowebshop.tricentis.com/build-your-cheap-own-computer</t>
         </is>
       </c>
+      <c r="M77" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to the Picture of Build your own cheap computer product details page, showing the product name and price.</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="72" customHeight="1">
       <c r="A78" s="5" t="inlineStr">
@@ -5613,6 +5982,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/newproducts to demowebshop.tricentis.com/build-your-cheap-own-computer</t>
         </is>
       </c>
+      <c r="M78" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to the Build your own cheap computer product details page, showing the product name and price.</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="72" customHeight="1">
       <c r="A79" s="5" t="inlineStr">
@@ -5681,6 +6055,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/newproducts to demowebshop.tricentis.com/simple-computer</t>
         </is>
       </c>
+      <c r="M79" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to the Picture of Simple Computer product details page, showing the product name and price.</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="72" customHeight="1">
       <c r="A80" s="5" t="inlineStr">
@@ -5749,6 +6128,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/newproducts to demowebshop.tricentis.com/simple-computer</t>
         </is>
       </c>
+      <c r="M80" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to the Simple Computer product details page, showing the product name and price.</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="72" customHeight="1">
       <c r="A81" s="5" t="inlineStr">
@@ -5817,6 +6201,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/newproducts to demowebshop.tricentis.com/build-your-own-expensive-computer-2</t>
         </is>
       </c>
+      <c r="M81" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to the Picture of Build your own expensive computer product details page, showing the product name and price.</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="72" customHeight="1">
       <c r="A82" s="5" t="inlineStr">
@@ -5885,6 +6274,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/newproducts to demowebshop.tricentis.com/build-your-own-expensive-computer-2</t>
         </is>
       </c>
+      <c r="M82" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to the Build your own expensive computer product details page, showing the product name and price.</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="72" customHeight="1">
       <c r="A83" s="5" t="inlineStr">
@@ -5953,6 +6347,11 @@
           <t>POST | 201 | https://demowebshop.tricentis.com/addproducttocart/catalog/81/1/1</t>
         </is>
       </c>
+      <c r="M83" s="6" t="inlineStr">
+        <is>
+          <t>The item is added to the shopping cart and a confirmation message appears, with the shopping cart count increasing by one.</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="72" customHeight="1">
       <c r="A84" s="5" t="inlineStr">
@@ -6017,6 +6416,11 @@
       <c r="L84" s="5" t="inlineStr">
         <is>
           <t>POST | 201 | https://demowebshop.tricentis.com/addproducttocart/catalog/80/1/1</t>
+        </is>
+      </c>
+      <c r="M84" s="6" t="inlineStr">
+        <is>
+          <t>The second item is added to the shopping cart and a confirmation message appears, with the shopping cart count increasing accordingly.</t>
         </is>
       </c>
     </row>
@@ -6089,6 +6493,11 @@
           <t>POST | 201 | https://demowebshop.tricentis.com/addproducttocart/catalog/75/1/1</t>
         </is>
       </c>
+      <c r="M85" s="6" t="inlineStr">
+        <is>
+          <t>The third item is added to the shopping cart and a confirmation message appears, with the shopping cart count increasing accordingly.</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="72" customHeight="1">
       <c r="A86" s="5" t="inlineStr">
@@ -6155,6 +6564,11 @@
       <c r="L86" s="5" t="inlineStr">
         <is>
           <t>POST | 201 | https://demowebshop.tricentis.com/addproducttocart/catalog/74/1/1</t>
+        </is>
+      </c>
+      <c r="M86" s="6" t="inlineStr">
+        <is>
+          <t>The fourth item is added to the shopping cart and a confirmation message appears, with the shopping cart count increasing accordingly.</t>
         </is>
       </c>
     </row>
@@ -6227,6 +6641,11 @@
       <c r="L87" s="5" t="inlineStr">
         <is>
           <t>POST | 201 | https://demowebshop.tricentis.com/subscribenewsletter</t>
+        </is>
+      </c>
+      <c r="M87" s="6" t="inlineStr">
+        <is>
+          <t>The newsletter subscription request is submitted and a confirmation message is displayed for the entered email address.</t>
         </is>
       </c>
     </row>
@@ -6302,6 +6721,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/newproducts to demowebshop.tricentis.com/</t>
         </is>
       </c>
+      <c r="M88" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to the Demo Web Shop home page.</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="72" customHeight="1">
       <c r="A89" s="5" t="inlineStr">
@@ -6370,6 +6794,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/newproducts to demowebshop.tricentis.com/newproducts</t>
         </is>
       </c>
+      <c r="M89" s="6" t="inlineStr">
+        <is>
+          <t>The textbox displays the entered value test and accepts the input without an error message.</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="72" customHeight="1">
       <c r="A90" s="5" t="inlineStr">
@@ -6439,6 +6868,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/newproducts to demowebshop.tricentis.com/newproducts</t>
         </is>
       </c>
+      <c r="M90" s="6" t="inlineStr">
+        <is>
+          <t>The second textbox displays the entered value test and accepts the input without an error message.</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="72" customHeight="1">
       <c r="A91" s="5" t="inlineStr">
@@ -6512,6 +6946,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/ to Not recorded</t>
         </is>
       </c>
+      <c r="M91" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to the Picture of Build your own computer product details page from the Demo Web Shop home page.</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="72" customHeight="1">
       <c r="A92" s="5" t="inlineStr">
@@ -6580,6 +7019,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/computers to demowebshop.tricentis.com/desktops</t>
         </is>
       </c>
+      <c r="M92" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to the Desktops category page, displaying the list of desktop products.</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="72" customHeight="1">
       <c r="A93" s="5" t="inlineStr">
@@ -6648,6 +7092,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/computers to demowebshop.tricentis.com/notebooks</t>
         </is>
       </c>
+      <c r="M93" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to the Notebooks category page, displaying the list of notebook products.</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="72" customHeight="1">
       <c r="A94" s="5" t="inlineStr">
@@ -6716,6 +7165,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/computers to demowebshop.tricentis.com/accessories</t>
         </is>
       </c>
+      <c r="M94" s="6" t="inlineStr">
+        <is>
+          <t>The Accessories category page loads, showing the Accessories heading and its product listings.</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="72" customHeight="1">
       <c r="A95" s="5" t="inlineStr">
@@ -6784,6 +7238,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/computers to demowebshop.tricentis.com/desktops</t>
         </is>
       </c>
+      <c r="M95" s="6" t="inlineStr">
+        <is>
+          <t>The Desktops category page loads, showing the Desktops heading and its product listings.</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="72" customHeight="1">
       <c r="A96" s="5" t="inlineStr">
@@ -6852,6 +7311,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/computers to demowebshop.tricentis.com/notebooks</t>
         </is>
       </c>
+      <c r="M96" s="6" t="inlineStr">
+        <is>
+          <t>The Notebooks category page loads, showing the Notebooks heading and its product listings.</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="72" customHeight="1">
       <c r="A97" s="5" t="inlineStr">
@@ -6920,6 +7384,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/computers to demowebshop.tricentis.com/accessories</t>
         </is>
       </c>
+      <c r="M97" s="6" t="inlineStr">
+        <is>
+          <t>The Accessories category page loads, showing the Accessories heading and its product listings.</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="72" customHeight="1">
       <c r="A98" s="5" t="inlineStr">
@@ -6988,6 +7457,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/computers to demowebshop.tricentis.com/notebooks</t>
         </is>
       </c>
+      <c r="M98" s="6" t="inlineStr">
+        <is>
+          <t>The Notebooks category page loads, showing the Notebooks heading and its product listings.</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="72" customHeight="1">
       <c r="A99" s="5" t="inlineStr">
@@ -7056,6 +7530,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/computers to demowebshop.tricentis.com/accessories</t>
         </is>
       </c>
+      <c r="M99" s="6" t="inlineStr">
+        <is>
+          <t>The Accessories category page loads, showing the Accessories heading and its product listings.</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="72" customHeight="1">
       <c r="A100" s="5" t="inlineStr">
@@ -7124,6 +7603,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/gift-cards to demowebshop.tricentis.com/5-virtual-gift-card</t>
         </is>
       </c>
+      <c r="M100" s="6" t="inlineStr">
+        <is>
+          <t>The product details page for the $5 Virtual Gift Card opens, showing its name and price.</t>
+        </is>
+      </c>
     </row>
     <row r="101" ht="72" customHeight="1">
       <c r="A101" s="5" t="inlineStr">
@@ -7192,6 +7676,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/gift-cards to demowebshop.tricentis.com/5-virtual-gift-card</t>
         </is>
       </c>
+      <c r="M101" s="6" t="inlineStr">
+        <is>
+          <t>The product details page for the $5 Virtual Gift Card opens, showing its name and price.</t>
+        </is>
+      </c>
     </row>
     <row r="102" ht="72" customHeight="1">
       <c r="A102" s="5" t="inlineStr">
@@ -7260,6 +7749,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/gift-cards to demowebshop.tricentis.com/50-physical-gift-card</t>
         </is>
       </c>
+      <c r="M102" s="6" t="inlineStr">
+        <is>
+          <t>The product details page for the $50 Physical Gift Card opens, showing its name and price.</t>
+        </is>
+      </c>
     </row>
     <row r="103" ht="72" customHeight="1">
       <c r="A103" s="5" t="inlineStr">
@@ -7328,6 +7822,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/gift-cards to demowebshop.tricentis.com/50-physical-gift-card</t>
         </is>
       </c>
+      <c r="M103" s="6" t="inlineStr">
+        <is>
+          <t>The product details page for the $50 Physical Gift Card opens, showing its name and price.</t>
+        </is>
+      </c>
     </row>
     <row r="104" ht="72" customHeight="1">
       <c r="A104" s="5" t="inlineStr">
@@ -7396,6 +7895,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/gift-cards to demowebshop.tricentis.com/25-virtual-gift-card</t>
         </is>
       </c>
+      <c r="M104" s="6" t="inlineStr">
+        <is>
+          <t>The product details page for the $25 Virtual Gift Card opens, showing its name and price.</t>
+        </is>
+      </c>
     </row>
     <row r="105" ht="72" customHeight="1">
       <c r="A105" s="5" t="inlineStr">
@@ -7464,6 +7968,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/gift-cards to demowebshop.tricentis.com/25-virtual-gift-card</t>
         </is>
       </c>
+      <c r="M105" s="6" t="inlineStr">
+        <is>
+          <t>The product details page for the $25 Virtual Gift Card opens, showing its name and price.</t>
+        </is>
+      </c>
     </row>
     <row r="106" ht="72" customHeight="1">
       <c r="A106" s="5" t="inlineStr">
@@ -7532,6 +8041,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/gift-cards to demowebshop.tricentis.com/100-physical-gift-card</t>
         </is>
       </c>
+      <c r="M106" s="6" t="inlineStr">
+        <is>
+          <t>The product details page for the $100 Physical Gift Card opens, showing its name and price.</t>
+        </is>
+      </c>
     </row>
     <row r="107" ht="72" customHeight="1">
       <c r="A107" s="5" t="inlineStr">
@@ -7600,6 +8114,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/gift-cards to demowebshop.tricentis.com/100-physical-gift-card</t>
         </is>
       </c>
+      <c r="M107" s="6" t="inlineStr">
+        <is>
+          <t>The product details page for the $100 Physical Gift Card opens, showing its name and price.</t>
+        </is>
+      </c>
     </row>
     <row r="108" ht="72" customHeight="1">
       <c r="A108" s="5" t="inlineStr">
@@ -7663,6 +8182,11 @@
       <c r="L108" s="5" t="inlineStr">
         <is>
           <t>Page | status not applicable | demowebshop.tricentis.com/gift-cards to demowebshop.tricentis.com/gift-cards</t>
+        </is>
+      </c>
+      <c r="M108" s="6" t="inlineStr">
+        <is>
+          <t>The gift cards listing switches to Grid view, displaying products in a grid layout.</t>
         </is>
       </c>
     </row>
@@ -7734,6 +8258,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/gift-cards to demowebshop.tricentis.com/gift-cards</t>
         </is>
       </c>
+      <c r="M109" s="6" t="inlineStr">
+        <is>
+          <t>The gift cards listing switches to List view, displaying products in a list layout.</t>
+        </is>
+      </c>
     </row>
     <row r="110" ht="72" customHeight="1">
       <c r="A110" s="5" t="inlineStr">
@@ -7800,6 +8329,11 @@
       <c r="L110" s="5" t="inlineStr">
         <is>
           <t>Page | status not applicable | demowebshop.tricentis.com/gift-cards to demowebshop.tricentis.com/gift-cards</t>
+        </is>
+      </c>
+      <c r="M110" s="6" t="inlineStr">
+        <is>
+          <t>The gift cards listing sorts by Position, and the Position option is shown as selected in the combobox.</t>
         </is>
       </c>
     </row>
@@ -7871,6 +8405,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/gift-cards to demowebshop.tricentis.com/gift-cards</t>
         </is>
       </c>
+      <c r="M111" s="6" t="inlineStr">
+        <is>
+          <t>The gift cards listing sorts by Name: A to Z, with products in alphabetical order and the option shown as selected in the combobox.</t>
+        </is>
+      </c>
     </row>
     <row r="112" ht="72" customHeight="1">
       <c r="A112" s="5" t="inlineStr">
@@ -7939,6 +8478,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/register to demowebshop.tricentis.com/register</t>
         </is>
       </c>
+      <c r="M112" s="6" t="inlineStr">
+        <is>
+          <t>The Male radio button is selected on the Register page.</t>
+        </is>
+      </c>
     </row>
     <row r="113" ht="72" customHeight="1">
       <c r="A113" s="5" t="inlineStr">
@@ -8008,6 +8552,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/register to demowebshop.tricentis.com/register</t>
         </is>
       </c>
+      <c r="M113" s="6" t="inlineStr">
+        <is>
+          <t>The Female radio button is selected and the Male radio button is cleared, since only one gender can be chosen.</t>
+        </is>
+      </c>
     </row>
     <row r="114" ht="72" customHeight="1">
       <c r="A114" s="5" t="inlineStr">
@@ -8067,6 +8616,11 @@
       <c r="L114" s="5" t="inlineStr">
         <is>
           <t>Page | status not applicable | demowebshop.tricentis.com/register to demowebshop.tricentis.com/register</t>
+        </is>
+      </c>
+      <c r="M114" s="6" t="inlineStr">
+        <is>
+          <t>The First name: field accepts the entered value and displays it in the textbox.</t>
         </is>
       </c>
     </row>
@@ -8129,6 +8683,11 @@
       <c r="L115" s="5" t="inlineStr">
         <is>
           <t>Page | status not applicable | demowebshop.tricentis.com/register to demowebshop.tricentis.com/register</t>
+        </is>
+      </c>
+      <c r="M115" s="6" t="inlineStr">
+        <is>
+          <t>The Last name: field accepts the entered value and displays it in the textbox.</t>
         </is>
       </c>
     </row>
@@ -8192,6 +8751,11 @@
       <c r="L116" s="5" t="inlineStr">
         <is>
           <t>Page | status not applicable | demowebshop.tricentis.com/register to demowebshop.tricentis.com/register</t>
+        </is>
+      </c>
+      <c r="M116" s="6" t="inlineStr">
+        <is>
+          <t>The Confirm password textbox accepts the tester-supplied value without an error, and the entered characters are masked rather than displayed as plain text.</t>
         </is>
       </c>
     </row>
@@ -8258,6 +8822,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/register to demowebshop.tricentis.com/register</t>
         </is>
       </c>
+      <c r="M117" s="6" t="inlineStr">
+        <is>
+          <t>The Email textbox accepts the tester-supplied value without an error message, and the entered value remains in the field.</t>
+        </is>
+      </c>
     </row>
     <row r="118" ht="72" customHeight="1">
       <c r="A118" s="5" t="inlineStr">
@@ -8315,6 +8884,11 @@
       <c r="L118" s="5" t="inlineStr">
         <is>
           <t>Page | status not applicable | demowebshop.tricentis.com/register to demowebshop.tricentis.com/register</t>
+        </is>
+      </c>
+      <c r="M118" s="6" t="inlineStr">
+        <is>
+          <t>The Password textbox accepts the tester-supplied value without an error, and the entered characters are masked rather than displayed as plain text.</t>
         </is>
       </c>
     </row>
@@ -8375,6 +8949,11 @@
       <c r="L119" s="5" t="inlineStr">
         <is>
           <t>Page | status not applicable | demowebshop.tricentis.com/register to demowebshop.tricentis.com/register</t>
+        </is>
+      </c>
+      <c r="M119" s="6" t="inlineStr">
+        <is>
+          <t>Clicking Register submits the registration form and the page displays a registration outcome, either a success confirmation or validation messages for any missing or invalid required fields.</t>
         </is>
       </c>
     </row>
@@ -8445,6 +9024,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/jewelry to demowebshop.tricentis.com/jewelry</t>
         </is>
       </c>
+      <c r="M120" s="6" t="inlineStr">
+        <is>
+          <t>Clicking the 0.00 - 500.00 price filter link updates the JEWELRY page so that only products priced within that range are listed.</t>
+        </is>
+      </c>
     </row>
     <row r="121" ht="72" customHeight="1">
       <c r="A121" s="5" t="inlineStr">
@@ -8513,6 +9097,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/jewelry to demowebshop.tricentis.com/jewelry</t>
         </is>
       </c>
+      <c r="M121" s="6" t="inlineStr">
+        <is>
+          <t>Clicking the 500.00 - 700.00 price filter link updates the JEWELRY page so that only products priced within that range are listed.</t>
+        </is>
+      </c>
     </row>
     <row r="122" ht="72" customHeight="1">
       <c r="A122" s="5" t="inlineStr">
@@ -8581,6 +9170,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/jewelry to demowebshop.tricentis.com/jewelry</t>
         </is>
       </c>
+      <c r="M122" s="6" t="inlineStr">
+        <is>
+          <t>Clicking the 700.00 - 3000.00 price filter link updates the JEWELRY page so that only products priced within that range are listed.</t>
+        </is>
+      </c>
     </row>
     <row r="123" ht="72" customHeight="1">
       <c r="A123" s="5" t="inlineStr">
@@ -8649,6 +9243,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/jewelry to demowebshop.tricentis.com/diamond-tennis-bracelet</t>
         </is>
       </c>
+      <c r="M123" s="6" t="inlineStr">
+        <is>
+          <t>Clicking the Picture of Diamond Tennis Bracelet opens the Diamond Tennis Bracelet product details page showing the product name, price, and Add to cart button.</t>
+        </is>
+      </c>
     </row>
     <row r="124" ht="72" customHeight="1">
       <c r="A124" s="5" t="inlineStr">
@@ -8717,6 +9316,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/jewelry to demowebshop.tricentis.com/diamond-tennis-bracelet</t>
         </is>
       </c>
+      <c r="M124" s="6" t="inlineStr">
+        <is>
+          <t>Clicking the Diamond Tennis Bracelet link opens the Diamond Tennis Bracelet product details page showing the product name, price, and Add to cart button.</t>
+        </is>
+      </c>
     </row>
     <row r="125" ht="72" customHeight="1">
       <c r="A125" s="5" t="inlineStr">
@@ -8785,6 +9389,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/jewelry to demowebshop.tricentis.com/vintage-style-three-stone-diamond-engagement-ring</t>
         </is>
       </c>
+      <c r="M125" s="6" t="inlineStr">
+        <is>
+          <t>Clicking the Picture of Vintage Style Three Stone Diamond Engagement Ring opens its product details page showing the product name, price, and Add to cart button.</t>
+        </is>
+      </c>
     </row>
     <row r="126" ht="72" customHeight="1">
       <c r="A126" s="5" t="inlineStr">
@@ -8853,6 +9462,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/jewelry to demowebshop.tricentis.com/vintage-style-three-stone-diamond-engagement-ring</t>
         </is>
       </c>
+      <c r="M126" s="6" t="inlineStr">
+        <is>
+          <t>Clicking the Vintage Style Three Stone Diamond Engagement Ring link opens its product details page showing the product name, price, and Add to cart button.</t>
+        </is>
+      </c>
     </row>
     <row r="127" ht="72" customHeight="1">
       <c r="A127" s="5" t="inlineStr">
@@ -8921,6 +9535,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/jewelry to demowebshop.tricentis.com/black-white-diamond-heart</t>
         </is>
       </c>
+      <c r="M127" s="6" t="inlineStr">
+        <is>
+          <t>Clicking the Picture of Black &amp; White Diamond Heart opens the Black &amp; White Diamond Heart product details page showing the product name, price, and Add to cart button.</t>
+        </is>
+      </c>
     </row>
     <row r="128" ht="72" customHeight="1">
       <c r="A128" s="5" t="inlineStr">
@@ -8989,6 +9608,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/jewelry to demowebshop.tricentis.com/black-white-diamond-heart</t>
         </is>
       </c>
+      <c r="M128" s="6" t="inlineStr">
+        <is>
+          <t>Clicking the Black &amp; White Diamond Heart link opens its product details page showing the product name, price, and Add to cart button.</t>
+        </is>
+      </c>
     </row>
     <row r="129" ht="72" customHeight="1">
       <c r="A129" s="5" t="inlineStr">
@@ -9057,6 +9681,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/jewelry to demowebshop.tricentis.com/diamond-pave-earrings</t>
         </is>
       </c>
+      <c r="M129" s="6" t="inlineStr">
+        <is>
+          <t>Clicking the Picture of Diamond Pave Earrings opens the Diamond Pave Earrings product details page showing the product name, price, and Add to cart button.</t>
+        </is>
+      </c>
     </row>
     <row r="130" ht="72" customHeight="1">
       <c r="A130" s="5" t="inlineStr">
@@ -9125,6 +9754,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/jewelry to demowebshop.tricentis.com/diamond-pave-earrings</t>
         </is>
       </c>
+      <c r="M130" s="6" t="inlineStr">
+        <is>
+          <t>Clicking the Diamond Pave Earrings link opens its product details page showing the product name, price, and Add to cart button.</t>
+        </is>
+      </c>
     </row>
     <row r="131" ht="72" customHeight="1">
       <c r="A131" s="5" t="inlineStr">
@@ -9193,6 +9827,11 @@
           <t>POST | 201 | https://demowebshop.tricentis.com/addproducttocart/catalog/71/1/1</t>
         </is>
       </c>
+      <c r="M131" s="6" t="inlineStr">
+        <is>
+          <t>Clicking Add to cart adds the product to the shopping cart, and the header cart count updates to reflect the added item.</t>
+        </is>
+      </c>
     </row>
     <row r="132" ht="72" customHeight="1">
       <c r="A132" s="5" t="inlineStr">
@@ -9262,6 +9901,11 @@
           <t>POST | 201 | https://demowebshop.tricentis.com/subscribenewsletter</t>
         </is>
       </c>
+      <c r="M132" s="6" t="inlineStr">
+        <is>
+          <t>Clicking Subscribe submits the newsletter subscription request and the page displays a confirmation or success message.</t>
+        </is>
+      </c>
     </row>
     <row r="133" ht="72" customHeight="1">
       <c r="A133" s="5" t="inlineStr">
@@ -9332,6 +9976,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/jewelry to demowebshop.tricentis.com/create-it-yourself-jewelry</t>
         </is>
       </c>
+      <c r="M133" s="6" t="inlineStr">
+        <is>
+          <t>Clicking the Picture of Create Your Own Jewelry opens the Create Your Own Jewelry page.</t>
+        </is>
+      </c>
     </row>
     <row r="134" ht="72" customHeight="1">
       <c r="A134" s="5" t="inlineStr">
@@ -9400,6 +10049,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/jewelry to demowebshop.tricentis.com/create-it-yourself-jewelry</t>
         </is>
       </c>
+      <c r="M134" s="6" t="inlineStr">
+        <is>
+          <t>Clicking the Create Your Own Jewelry link opens the Create Your Own Jewelry page.</t>
+        </is>
+      </c>
     </row>
     <row r="135" ht="72" customHeight="1">
       <c r="A135" s="5" t="inlineStr">
@@ -9463,6 +10117,11 @@
       <c r="L135" s="5" t="inlineStr">
         <is>
           <t>Page | status not applicable | demowebshop.tricentis.com/jewelry to demowebshop.tricentis.com/jewelry</t>
+        </is>
+      </c>
+      <c r="M135" s="6" t="inlineStr">
+        <is>
+          <t>Selecting Grid in the combobox changes the JEWELRY product listing to grid view.</t>
         </is>
       </c>
     </row>
@@ -9533,6 +10192,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/blog to demowebshop.tricentis.com/blog/month/2014-7</t>
         </is>
       </c>
+      <c r="M136" s="6" t="inlineStr">
+        <is>
+          <t>Clicking the July (2) link opens the blog month page listing blog posts from July 2014.</t>
+        </is>
+      </c>
     </row>
     <row r="137" ht="72" customHeight="1">
       <c r="A137" s="5" t="inlineStr">
@@ -9597,6 +10261,11 @@
       <c r="L137" s="5" t="inlineStr">
         <is>
           <t>Page | status not applicable | demowebshop.tricentis.com/blog to demowebshop.tricentis.com/blog/tag/asp.net</t>
+        </is>
+      </c>
+      <c r="M137" s="6" t="inlineStr">
+        <is>
+          <t>Clicking the asp.net link opens the blog tag page listing blog posts tagged asp.net.</t>
         </is>
       </c>
     </row>
@@ -9667,6 +10336,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/blog to demowebshop.tricentis.com/blog/tag/e-commerce</t>
         </is>
       </c>
+      <c r="M138" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to the 'e-commerce' tag page under the Blog section, and the page lists blog posts tagged 'e-commerce'.</t>
+        </is>
+      </c>
     </row>
     <row r="139" ht="72" customHeight="1">
       <c r="A139" s="5" t="inlineStr">
@@ -9735,6 +10409,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/blog to demowebshop.tricentis.com/blog/tag/money</t>
         </is>
       </c>
+      <c r="M139" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to the 'money' tag page under the Blog section, and the page lists blog posts tagged 'money'.</t>
+        </is>
+      </c>
     </row>
     <row r="140" ht="72" customHeight="1">
       <c r="A140" s="5" t="inlineStr">
@@ -9803,6 +10482,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/blog to demowebshop.tricentis.com/blog/tag/sample%20tag</t>
         </is>
       </c>
+      <c r="M140" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to the 'sample tag' tag page under the Blog section, and the page lists blog posts tagged 'sample tag'.</t>
+        </is>
+      </c>
     </row>
     <row r="141" ht="72" customHeight="1">
       <c r="A141" s="5" t="inlineStr">
@@ -9866,6 +10550,11 @@
       <c r="L141" s="5" t="inlineStr">
         <is>
           <t>Page | status not applicable | demowebshop.tricentis.com/blog to Not recorded</t>
+        </is>
+      </c>
+      <c r="M141" s="6" t="inlineStr">
+        <is>
+          <t>The 'Customer Service - Client Service' blog post opens, displaying its title and content.</t>
         </is>
       </c>
     </row>
@@ -9936,6 +10625,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/blog to demowebshop.tricentis.com/blog/tag/sample%20tag</t>
         </is>
       </c>
+      <c r="M142" s="6" t="inlineStr">
+        <is>
+          <t>The browser navigates to the 'sample tag' tag page under the Blog section, and the page lists blog posts tagged 'sample tag'.</t>
+        </is>
+      </c>
     </row>
     <row r="143" ht="72" customHeight="1">
       <c r="A143" s="5" t="inlineStr">
@@ -10006,6 +10700,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/blog to Not recorded</t>
         </is>
       </c>
+      <c r="M143" s="6" t="inlineStr">
+        <is>
+          <t>The comments section of the selected blog post is displayed, showing the comments for that post.</t>
+        </is>
+      </c>
     </row>
     <row r="144" ht="72" customHeight="1">
       <c r="A144" s="5" t="inlineStr">
@@ -10074,6 +10773,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/apparel-shoes to demowebshop.tricentis.com/genuine-leather-handbag-with-cell-phone-holder-many-pockets</t>
         </is>
       </c>
+      <c r="M144" s="6" t="inlineStr">
+        <is>
+          <t>The product details page for 'Picture of Genuine Leather Handbag with Cell Phone Holder &amp; Many Pockets' opens, showing the product name, price, and an Add to cart option.</t>
+        </is>
+      </c>
     </row>
     <row r="145" ht="72" customHeight="1">
       <c r="A145" s="5" t="inlineStr">
@@ -10142,6 +10846,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/apparel-shoes to demowebshop.tricentis.com/genuine-leather-handbag-with-cell-phone-holder-many-pockets</t>
         </is>
       </c>
+      <c r="M145" s="6" t="inlineStr">
+        <is>
+          <t>The product details page for 'Genuine Leather Handbag with Cell Phone Holder &amp; Many Pockets' opens, showing the product name, price, and an Add to cart option.</t>
+        </is>
+      </c>
     </row>
     <row r="146" ht="72" customHeight="1">
       <c r="A146" s="5" t="inlineStr">
@@ -10210,6 +10919,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/apparel-shoes to demowebshop.tricentis.com/green-and-blue-sneaker</t>
         </is>
       </c>
+      <c r="M146" s="6" t="inlineStr">
+        <is>
+          <t>The product details page for 'Picture of Green and blue Sneaker' opens, showing the product name, price, and an Add to cart option.</t>
+        </is>
+      </c>
     </row>
     <row r="147" ht="72" customHeight="1">
       <c r="A147" s="5" t="inlineStr">
@@ -10278,6 +10992,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/apparel-shoes to demowebshop.tricentis.com/green-and-blue-sneaker</t>
         </is>
       </c>
+      <c r="M147" s="6" t="inlineStr">
+        <is>
+          <t>The product details page for 'Green and blue Sneaker' opens, showing the product name, price, and an Add to cart option.</t>
+        </is>
+      </c>
     </row>
     <row r="148" ht="72" customHeight="1">
       <c r="A148" s="5" t="inlineStr">
@@ -10346,6 +11065,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/apparel-shoes to demowebshop.tricentis.com/50s-rockabilly-polka-dot-top-jr-plus-size</t>
         </is>
       </c>
+      <c r="M148" s="6" t="inlineStr">
+        <is>
+          <t>The product details page for 'Picture of 50's Rockabilly Polka Dot Top JR Plus Size' opens, showing the product name, price, and an Add to cart option.</t>
+        </is>
+      </c>
     </row>
     <row r="149" ht="72" customHeight="1">
       <c r="A149" s="5" t="inlineStr">
@@ -10414,6 +11138,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/apparel-shoes to demowebshop.tricentis.com/50s-rockabilly-polka-dot-top-jr-plus-size</t>
         </is>
       </c>
+      <c r="M149" s="6" t="inlineStr">
+        <is>
+          <t>The product details page for '50's Rockabilly Polka Dot Top JR Plus Size' opens, showing the product name, price, and an Add to cart option.</t>
+        </is>
+      </c>
     </row>
     <row r="150" ht="72" customHeight="1">
       <c r="A150" s="5" t="inlineStr">
@@ -10482,6 +11211,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/apparel-shoes to demowebshop.tricentis.com/casual-belt</t>
         </is>
       </c>
+      <c r="M150" s="6" t="inlineStr">
+        <is>
+          <t>The product details page for 'Picture of Casual Golf Belt' opens, showing the product name, price, and an Add to cart option.</t>
+        </is>
+      </c>
     </row>
     <row r="151" ht="72" customHeight="1">
       <c r="A151" s="5" t="inlineStr">
@@ -10550,6 +11284,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/apparel-shoes to demowebshop.tricentis.com/casual-belt</t>
         </is>
       </c>
+      <c r="M151" s="6" t="inlineStr">
+        <is>
+          <t>The product details page for 'Casual Golf Belt' opens, showing the product name, price, and an Add to cart option.</t>
+        </is>
+      </c>
     </row>
     <row r="152" ht="72" customHeight="1">
       <c r="A152" s="5" t="inlineStr">
@@ -10618,6 +11357,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/apparel-shoes to demowebshop.tricentis.com/custom-t-shirt</t>
         </is>
       </c>
+      <c r="M152" s="6" t="inlineStr">
+        <is>
+          <t>The product details page for 'Picture of Custom T-Shirt' opens, showing the product name, price, and an Add to cart option.</t>
+        </is>
+      </c>
     </row>
     <row r="153" ht="72" customHeight="1">
       <c r="A153" s="5" t="inlineStr">
@@ -10686,6 +11430,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/apparel-shoes to demowebshop.tricentis.com/custom-t-shirt</t>
         </is>
       </c>
+      <c r="M153" s="6" t="inlineStr">
+        <is>
+          <t>The product details page for 'Custom T-Shirt' opens, showing the product name, price, and an Add to cart option.</t>
+        </is>
+      </c>
     </row>
     <row r="154" ht="72" customHeight="1">
       <c r="A154" s="5" t="inlineStr">
@@ -10754,6 +11503,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/apparel-shoes to demowebshop.tricentis.com/apparel-shoes</t>
         </is>
       </c>
+      <c r="M154" s="6" t="inlineStr">
+        <is>
+          <t>The apparel and shoes category listing shows page 2 of products, with the page URL remaining on the apparel-shoes category.</t>
+        </is>
+      </c>
     </row>
     <row r="155" ht="72" customHeight="1">
       <c r="A155" s="5" t="inlineStr">
@@ -10822,6 +11576,11 @@
           <t>Page | status not applicable | demowebshop.tricentis.com/apparel-shoes to demowebshop.tricentis.com/apparel-shoes</t>
         </is>
       </c>
+      <c r="M155" s="6" t="inlineStr">
+        <is>
+          <t>The apparel and shoes category listing advances to the next page of products, with the page URL remaining on the apparel-shoes category.</t>
+        </is>
+      </c>
     </row>
     <row r="156" ht="72" customHeight="1">
       <c r="A156" s="5" t="inlineStr">
@@ -10888,6 +11647,11 @@
       <c r="L156" s="5" t="inlineStr">
         <is>
           <t>Page | status not applicable | demowebshop.tricentis.com/apparel-shoes to demowebshop.tricentis.com/v-blue-juniors-cuffed-denim-short-with-rhinestones</t>
+        </is>
+      </c>
+      <c r="M156" s="6" t="inlineStr">
+        <is>
+          <t>The product details page for 'Picture of Denim Short with Rhinestones' opens, showing the product name, price, and an Add to cart option.</t>
         </is>
       </c>
     </row>
@@ -10983,7 +11747,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>445734641b7c5653acd01dee3b9fc4197b07574f3e10b80bf27212c3575deadb</t>
+          <t>29d7915253a550d38492337df4de10514b8c3d9fbae30d0118a8366876f09702</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -11017,7 +11781,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>b3badc01dc30f1b49cbe34cacf83e1699da56c4364b6191d5b4a5d96450ad471</t>
+          <t>a7042562df37de8d941fc48c6d3c8c2dc64af10cd020e457a48d8f8720f00216</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -11051,7 +11815,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>181c48ac2daf7224612d16d74f49725e11f3ced6dc19690e3601edfa4de6106b</t>
+          <t>c0fe89db07d406d4ef6919d562760d91d71d0ecc60769fa0408387ba13734f36</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -11085,7 +11849,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>24c9dbbd9b058d6666b8bdf1b5901dc496172d83bbec403e2bc9e72b126487e0</t>
+          <t>1d58296fd58002f92887479b857b50f0882098b6da308a8a8250e8a259e90f48</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -11119,7 +11883,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>49ebb2dbe3a52b6a6d76ea4bc49b8aff9c544545a4d0d65abdb8cde0147a7edb</t>
+          <t>a599987d36f467b0fb21e621473fb23d5cfbb0bd1272bdbdb94b6582c2ac0de6</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -11153,7 +11917,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>a1aa5187058d941919834b5a230b9d028f4ec984ebaef47ac477e04fc7b64e07</t>
+          <t>0d38284354364f5bd0bf59fe033dca1c9be04ba876f02e8ba7f4536130ebc451</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -11187,7 +11951,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>1124536a778edb88f99a8e111c17c3c0394dae9b9bbc239b6010f75cc6f0f09a</t>
+          <t>5e66656691a979ea00c0fb5de05c5f169ec143bcdfe0c7d8bc644f5e46c9386f</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -11221,7 +11985,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2cfa0f518d4e72d62e6989948b6f6b99f78dc044995e8948c96e7f5f33d42bb9</t>
+          <t>cab67df6bb4c0fe48e9bbbb53ec52645198718b9887b3345c8ace8c88e60b539</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -11255,7 +12019,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>d5d77d61acf9c9750bf624b6aa6cd77dd1bf8b5391beb0432062a67faf5b8522</t>
+          <t>9bbd528809a63078a785c9ba5444abde248cc70d004c4eae4280eafac845055a</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -11289,7 +12053,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>0c79e627ece279a610dd139095ec3ee2c7979e1186d5a5a4c4d439e4feff4f10</t>
+          <t>1b214936b258d2970013cb2acb612cb0f4730975d4094f8002a9a293c0e60d7e</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -11323,7 +12087,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>b23af3956315be1515076561039f2eabb376147eb0d7dd3f041b49485455a7ea</t>
+          <t>b90a0875f8681cbdc9f35d4108d060244aa656c1a9f6b1d81ffe44ce658283a0</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -11357,7 +12121,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>4a6d23e8ffd0a029155f97a300f3b55a8b781a60cbede9c73ad4f65113479923</t>
+          <t>ba8c31b259733a14ed70908cf763cfd85aec96947bb5a2d08422304066632a0a</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -11391,7 +12155,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>4d04ddfe0e3b8bb1e3522bc6f7793f2e4fe0d223852ea7fd3d1f4e696c72954d</t>
+          <t>26c23ec9eea8a435c7be1c50b9cb33f483bd0200adcd92190dc25ac0749230c3</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -11425,7 +12189,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>7e4cf78ae99e74bbcb75f78cb62d4df941ddc3b3483478b8f8c0ce82b9014e6f</t>
+          <t>b0beb85a2b1f5b4c07a120869cbeee6c7bc95515f0aed125c4e1993c90802602</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -11459,7 +12223,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>62c64d1413d7a77f18cc285a3aceded621a364b163c22c7ccd3463e13d6c8782</t>
+          <t>5c63e77a030cfff98d352dc2081666ae6d4165e27090b554d1ab46a835476d7c</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -11493,7 +12257,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>09ff896641492346e3c2f023fd6278a9a0e0b7ec208c9183720a7b730b20bbbf</t>
+          <t>df0c0851ee50663c7f0088bc89d2c3eea58eb113fe90a23ac8ea9dfe12205513</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -11527,7 +12291,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>4fe16719879680ca6bb1b153e2222f32a1e7b219c689f8d11192102f471e0e38</t>
+          <t>8035169274cd5efe2ab442c66a8d36e8937e4bf18d0c34277aa7ce2ad46f407d</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -11561,7 +12325,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>bccdf2a8306e3cd7e32477eea2bea2c908736ff7f53000f957311dba27ca7569</t>
+          <t>b74af78b7ca5c6363b7cf91e4cf81548667b430db1fbd46a6d788ba4f7199814</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -11595,7 +12359,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>a75b4dc2260c3b7e6f9bc86cf84d3c916b2e30d29a30f711c7c8bba4a8f71a8e</t>
+          <t>292c64b14f9aaf825143039d5543d9cf2d8edeb36066b8dbf9637127e34c6f8b</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -11629,7 +12393,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>76a6caec8e13782b03f68a5ffe0b27197ff3e93c99e4c5e66e28a91a3fc4d8c9</t>
+          <t>36ed56a64cfd582c4b8d4db79aa99fea971281f4560147fe128af14cb5dbf4f9</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -11663,7 +12427,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>eb042e237c2b326eb1dc67e6a2e429c1cb7929ca7580d6c978c74b538bfe6780</t>
+          <t>602807fafa2e18ef6b61f737468e26f1674ad3fff5c07039fad792c40df9e781</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -11697,7 +12461,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>148afa6dfb2b12f24b3c5a840a65c15d2a735a43ddce526b08b1e6ca5f2d4d0a</t>
+          <t>6b021d72f3d9602cd4b8e821ef9363491fc25ff97b9d7e0320907fe71654b09c</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -11731,7 +12495,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>b59622bd3d6398ea2326b149abee0939f3459d840e8afa5b1256f4aaed04bb05</t>
+          <t>423701f5fb45fb7d90d95d9c4bfc4edee5e9edb9e2d7dd8d3751b7a9fd5264da</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -11765,7 +12529,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>4adaa79d5c6993b9cbc3baa8f28e5d3ff986d30a617c01795775faadc893f72e</t>
+          <t>b2b00598557b49d914d87828497795ec7ce9a97d185bbceaa158fc1f22e187ab</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -11799,7 +12563,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>4ac450c965225cd81f11098af8700be17ddc5d3d6a99803008c3b172e0918872</t>
+          <t>c3aa156326616a2cfbd4024d7a615dda6562cf2d8a95a97ae14f3d7d6a0a659d</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -11833,7 +12597,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>84699065be2f128b41b50cd2365d82b5269a5c342551350c72408adbfe0203a5</t>
+          <t>36ac7a2e2d2db978db75ff36f3079b46a7cb98ca5f706895825d50d890e7fdbc</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -11867,7 +12631,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>4fcb3e8c3a320b11323f1275e3cc7bd5d2edc042e08ad282bd8bc8dcb384f99d</t>
+          <t>b9d5473ef1419f4ef24eee72d513d675312f7a82f07d1c4a910e869dc5b0a6c4</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -11901,7 +12665,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>8a1401df3752f7cb0923d35952529ca615b758066d7576de3b81f2bc21ad2823</t>
+          <t>8420c4fb83cf8baddd59d1566d57ca2c2ab7613f00f98e21f6e39ec0607afdd3</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -11935,7 +12699,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>8c73f0c20cf8125107bfdd43f2267e6af40962ccf580be2a05274dbfe2706fac</t>
+          <t>df05c551e0459ebf4ffbf9195f216fac1358b76c787207083e67037f6a4239de</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -11969,7 +12733,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>bf100aae1286a2b8a7040d6c1582408510e1eabfad62dd1db96c1780f5fdd000</t>
+          <t>02b9ede541cd1375d0b389e473bf480896e5e4500f04442735a6e125af3709a6</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -12003,7 +12767,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>45415639898e1b62341c9dd81074733bffe127ba8e372d9cf2a6ab9761232d7e</t>
+          <t>c0639f28474dd0af2a14d8e9fa729cefa0d58d35dd30f0d1d114df370b9be6ad</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -12037,7 +12801,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>12878ff18baf922af0ecb5d8a58685238752f699ff3e2625afad603393db8ebe</t>
+          <t>e86bc80ae2c881b3508c381b2e139017eb7c7a1066b1e273b436e10dbc96f933</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -12071,7 +12835,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>cae7f5aa12c3d41d13ac6c7c88ccecf1d921790a501bdbd7b93ef1deffc5e34e</t>
+          <t>22570003e88392e18f0c28e7ac63f74c71988d87b049dcd1097533c30387905e</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -12105,7 +12869,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>27338cc53f69f4078991479e6b4aa6e95b36ca81d71559fc3d7ac37eff6956c3</t>
+          <t>d1fb9793fdcbdd1a70f81d8f4eb000d8356fd1090753c55afaa15d6f3ea28aff</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -12139,7 +12903,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2929a86f5470635eb92cca86d5ebbee27008bd52c280b1ae03a0c9e4613cda91</t>
+          <t>7c6b6b15280aae7d9ac3c95548d921c85765de0cf5b8fc29ae65d7944997f19b</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -12173,7 +12937,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>d75aae8adbe14a04e1098cf90a36beaefeda1c23af32241d495513ecb4b74b49</t>
+          <t>85a27cd366970f6cff0f7bd51a0ed06bb46e5b50c8e0c3a577f7416ee3e91586</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -12207,7 +12971,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>d4d7b8a39bab792d5d3f2c872fee3a4fdcf4cb141c93cb9534d784f1130a2c40</t>
+          <t>2360babe4ec4f520fea1e1b06887c9c79b656879e216142bb3a7858aec3af304</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -12241,7 +13005,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>12278fe79cb0fbc94702c00e3436f47c93113890d1d82d01893b811e9e866b60</t>
+          <t>e14d1f139833a9eadc1068259c4f6740da94451123c13bf975a09d2913ba4b8d</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -12275,7 +13039,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>045abab9be40da1dfee87990c561bdeffbf1778cbdd0ad7e5c5b9996fb276a3f</t>
+          <t>31a609ea736dcf09179e7834aa1a1d4130ee94cbfa327f92f8d0ed1542713c56</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -12309,7 +13073,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>9f137319ad28448571e0b637912804bea8fb75bca6dc2d7555a2f4668f1c1bee</t>
+          <t>d56bb050fc0f92e341fbf55087cbfcf290c961d2d62e095571f058e1f0b28296</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -12343,7 +13107,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2937d542441431c84305bee887aa513f5437a026c64583f152d9cde8dd6aacde</t>
+          <t>417710e0b285bdb775374133134683d53c8ab7f4acbc18980588c2a6a666473c</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -12377,7 +13141,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>73e5c990a4447fee5508c957e98913728c0abc4af926c81db38339672384d84c</t>
+          <t>fbb56bc678b232e2252f0bd3930e95bbe7f0484c7d8ef1740b15defe83e7bd60</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -12411,7 +13175,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>a0f6e4ae8a284bce35fa4abfab1c82102b1e15fa45c5702b42d8428dcd2afae1</t>
+          <t>fd65f7e24224cd3c975cbe62c1098de7e1dfb463f3e77cde83a0c35e225d0b59</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -12445,7 +13209,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>903f72cdcb88f1e6817671f3114c113a7c63f8edce0ae1513dda07ba7787c545</t>
+          <t>8b3d8642239606bba627e31a63396a00334bcd238b63c857c1cd472a6856378c</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -12479,7 +13243,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>f408a2049573261f267c212a047f0da37fbebdfba088cee1c92831ad1f51ef55</t>
+          <t>f75c6246638c550e841a27bdb355b040c37fd8b848f678600c1af2b281072703</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -12513,7 +13277,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>3d30fa82d1ea5ad22abae9291f6fdd03ca0d649e0e6888d28efc121ec3e0823c</t>
+          <t>824b42f87fafb72eaa200f75d32581a7666f598e44aa0b6c042717ee06f62eff</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -12547,7 +13311,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>202066d60c658c1aa309b5ca7e4d874587f6e09642bce6b5551ddb34ecf3b146</t>
+          <t>9ecc88afc1def2dd04b3c94c4f9e499eda0476be347f3fa616ae8722e9f0ee82</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -12581,7 +13345,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>a2c68f57201f38b2504252c90e43eb8e87e927f008a3362fe761816403e9505c</t>
+          <t>9adc78c9d6c2ec13b5941c0ff099b3eb65e6a186ec25ac9fe6ccd752a83454aa</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -12615,7 +13379,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>3eba29b518069a999d993cd426532fddafcccec6ee0f821ce8e42d0c3a43c44f</t>
+          <t>d6a4557bd1a7d7312652c0d62c8b7d2edc10a59bddd83c5a225207a73bdb0a5c</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -12649,7 +13413,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>4d0e38a43f928e6c9594538b68eff1099c7273cfda771c574ab7474a548fc678</t>
+          <t>b91b5b31ef69686f80ecf2c293b7f801721684412490331d4e3bdb2d48243356</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -12683,7 +13447,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>d650b057aabb1ffa90d9d1235e06ffdc4fa9d213ac45b75b2c049a99232aa914</t>
+          <t>3dee168f52abaea8b5f36f275aa83b5982567ebe042fab1a51f019eb9d872dc4</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -12717,7 +13481,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>c0af89c53634fd17b7f5e6fecc8cbae2be1ceac0ce45f7e280e6eeb9672fc81b</t>
+          <t>d77e6c97381ab689914ac701e89ae40e349d06416821ee6ecb46abc626ca51a7</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -12751,7 +13515,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>7e133210fbde6e16127171a65b6ee149ab4f2978be2cf843cd51d5a6698d9b93</t>
+          <t>e2626635f7625ac979498e00ae88650887f37918e69feb224ec7909de82f7d7f</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -12785,7 +13549,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>79b79d782c68f86515f362f6bd113ff52c49fa621c2e67d65be519956135a0f5</t>
+          <t>50e413beea882cb860ca96c7ed98f4df13fe2a24397391ed1ad59e917ebd0362</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -12819,7 +13583,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>ddd6a81f28bf78150b728013b99a10fd27993b7e6e2bbf2ca0cd8d64ad4503cb</t>
+          <t>ec27150bd3b7da9bf7fb6178abddebf2114b88c8d160c3c1abaf5aea250bba0b</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -12853,7 +13617,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>55dcadde8acd8ddf915f595ce17e5e4b2e4e1c2fff3c1a6ccd60ee9a8b516366</t>
+          <t>9d1fe12829eb9e3b744d41e1f776bbf645dbca05518161a07ceb6d52ebcf61be</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -12887,7 +13651,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>1a055e2bad2c9b5335dbc6cf72a387ea091ae12eb431c27745d0a0c782370af2</t>
+          <t>1cce571b177c7bf9cd936f554e2aedb717c33ac91300531e192aa80a8391f9db</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -12921,7 +13685,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>189d55149c9284c8eabc31887a9258c89679d063d247612aff81ff32208a9af8</t>
+          <t>5c5c85705cfefd9ef4d7f911cd5b43ccec51c6e9d1ccf6fb689f301ea1ab80d6</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -12955,7 +13719,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>db0ddfb1162e1e4699ba730be0254caec1d6263e7511959341e4e01d303a532d</t>
+          <t>7cfb757786731696e8585996acb7bf61e4e2cf562383afc4f8817435ac5bc2f4</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -12989,7 +13753,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>8c3cf3005f6c3a54e7ce9b1155527ea69bcfd61c8cd44a859b791b3fbbc6670b</t>
+          <t>62e6600b9eaa40f510732432a7fad56483c6ddfcc06d434fa97be23e1887e212</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -13023,7 +13787,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>95551c0e05e09537e89d104c08f9c26bfc2f478f82e3d97b73cfb595c30c6cb0</t>
+          <t>a8979a1e8a90a9c5ac8a2c0af8608ffa33769315dfa981a7fce5b55ee881e45d</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -13057,7 +13821,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>343e75d223b821961e6af84fb09660ab47b868ad877518e777682ee894af099c</t>
+          <t>ffaee5461fc5dfb9036cfdc8555a9044f83bc239e14d368ae0337072b82d3f2d</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -13091,7 +13855,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>4480c5adfb0def5a98857bb2e8f2f1fb7256c91c124141456248795739f781c0</t>
+          <t>11611752d133cb1317d94a25651c36fe508023c98bedf5ab49c04fdd097dff0d</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -13125,7 +13889,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>fb82eb5d9a8c44e2a764e84196ceef98ba220d583cce5d32b85ab1effbc93821</t>
+          <t>00e89fb95ac69da745a7dcbf7f1da2819f9d665a1c6b21db5e78942f63e3050c</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -13159,7 +13923,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>16de36f09ef52ddeca06fbc53b892eea0bd443b69e2545132137eac41f2e5696</t>
+          <t>24d03a0a3510098675924fe5dcf06be244d84e901a142220d944ec624c82ebd0</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -13193,7 +13957,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>a53751553485acfa13cf7d8bf82401b244198943dd1b2538ecb10180c99bf720</t>
+          <t>48cc2c48d39b134fd8daecfeb9d866bcfa912cd4e96f0d14a610bbde6395e889</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -13227,7 +13991,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>bdbe549b6f43cbf7380a1f84400d494be04555ce2df70826a7cd7606b9331cdc</t>
+          <t>22bc1476efd8bbc0b976e2b5345c8959f9d083b758dc0e68c7d19e63b8ce550a</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -13261,7 +14025,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>d2b10c27199d063ef1074fb8a241724bcc460051da170c3504b0baf7d30d0a11</t>
+          <t>856c7c51873e8256a5c7a42f07b4e04407fb64c5eda3535e9103136505739bd2</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -13295,7 +14059,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>8abb5f639de90e0b8998f3b4c724b40456396f23a88e1c6c908621a034746294</t>
+          <t>43bdfad9dea134ecdc70e86e0c2296747c75d5d807075442b6f4f90877771894</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -13329,7 +14093,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>a93ee01e8b2ba9cb745bfffe404c4a68d29a50c3b00e640bdfbfa7773ad74578</t>
+          <t>bd19151f9a40352918412f3800a6c023d25d506c8f7e48f42b1ed45631db25a8</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -13363,7 +14127,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>a8e516b5f89ce63e2a44cc7ce59be9481cdf7a66dc4d2fe2a2bf59f9c3feaeab</t>
+          <t>4ac20e1184a321ae07e621059dbedfc399c34b7a13cf8367aa3e6a4509be802d</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -13397,7 +14161,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>6c3e9fb704ccf7eee9398cb205cec32ccb17ed7db6428a3d1df9cfb49a021144</t>
+          <t>a2827e0ed54a0fbf0df2ceb2e034a9018a2d71362d1f45057c3612dcbaf20b83</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -13431,7 +14195,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>f2111422fd5aa0ebebb6e24c918d7baedd53354f3454dc877ef3b70ac727bf63</t>
+          <t>32f60620f5b520893156f55dd55fc59bfde1b6323e50be644fdd924297b87ae2</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -13465,7 +14229,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>129772e86e32bf5ce6dc430cff03d35d72fcb59811cdd203c09bde0d07b02f99</t>
+          <t>2a653120d3a17004d3dffd97be5495e76e2fe45fdd64f879d8eff45b7059027a</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -13499,7 +14263,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>10956e02707e254535e79f26871411554cd5ccc9eced9111d1475b33df075e3e</t>
+          <t>65a64dc5421eb7cdc70bc315cadcacf252f84d18cbfe07460effac8dcc1db98b</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -13533,7 +14297,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>29e8bf24e3512d521c7f51fad770a91aafd4e30fca17c3c905db1441416f06b2</t>
+          <t>f21e8f41cdb48387ef2ba08956c470551922b1029d29d0d7ad05b794f923bff8</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -13567,7 +14331,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>c8b256b755bf74a015024eea33140d13b4391c9de87c82c669b56ab66568fe5f</t>
+          <t>2325d7cde61f7ae7cc3456551527eabae11c79722e50dccdd3f5b8d0f56c0422</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -13601,7 +14365,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>c9288ae9f3092e50e455e998b173031fd90349b57616228c4928f4e9a8bf1ec5</t>
+          <t>8e86a40511873058b6a475eb9ac21dc47c0bef5f2b7c5d54170392a2655a5301</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -13635,7 +14399,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>4d4e4562bb06f6d18ce6dbf695b903936ecc95084f697419e88ba05ffed96480</t>
+          <t>cd1cdbe57f5d2ca6a501f83c051c84363d2fb9db6b57b8b80d18c9a40cdfec32</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -13669,7 +14433,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>0357b0f3e60df73ab05706478422dd9da6ea0baf5cf6876d1bba72c53434359d</t>
+          <t>f28907eb09a6fee22760aa0f12e13e423e8baaa2bb318b53c93e3364b71ce5e4</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -13703,7 +14467,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>80e81464f096d52bb46dcfce40f843b5b6e852cab6b549cb0e5dd178a408cab9</t>
+          <t>9ea802b5d971806f02cdd3fcce9e2f03d9094d18b2a54c5b85f18915efe76639</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -13737,7 +14501,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>543ae0f561529c39345917706f6c8864f86e96139d8386489e487be96459a9ac</t>
+          <t>d4b9ddf133d1c51cebecc4107aebb836c4adb2abdd5ed0e76558aac156c80f33</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -13771,7 +14535,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>a463b46437fb05b93af2e07f7ac364a5b9b7d9354b9790a34a2bf1a52269435e</t>
+          <t>8c738c4b09a89024e15df4b0f49a8a4224cad9f0d7da6f0ec9815b161b530874</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -13805,7 +14569,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>6246d9480702d03120829a8891b656e98f65f9443283f7bf2aad7f6f68ecd68f</t>
+          <t>c8f60e26bb77982aaa218e679358c1d4a6b0d916b17e08ce9b7f35f351a58380</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -13839,7 +14603,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>b0bc8c169dc968d2290d0128fc1fbdac5f9af4b7b806f73d42b8a52ac7e70d1b</t>
+          <t>c93cb6da24b14e5c62ba04ce4503e69e90c568e82707aeca59498a722f1d014a</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -13873,7 +14637,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>13f86e06deb7faf99e7cdfac7fd3d5da79894b9c10699d486299a71002b2e44b</t>
+          <t>84eb711eaffd1ddd865ef47e25814f6c2c4aed0b08b534313d83c8cfe454357a</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -13907,7 +14671,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>8afd6221bb74ce633291180b0e6b9dbb8d7e0c08be91d1cdb133e80f4919fca7</t>
+          <t>b31b707152aa8d648145745ab765530ab58fc5549dd515cefa4a1dd7cf3fa5ca</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -13941,7 +14705,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>49be0a81470dfed2275999a83cf6560bb538e34899d28eb58587bc39ffeee70b</t>
+          <t>48a42fea0a79fdc90f36e61834444224b4ca530276ea734417bbce3277886cc1</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -13975,7 +14739,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>2da09d1dc752d2a0c1b27a88b6db0d0a9bb4edbce87d37889145bba4f418c132</t>
+          <t>00ff5f1b3fbbae85961d866bd5de3e44ee615376f60c168789a13bf8c2d0e062</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -14009,7 +14773,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>e387a5a7de81d33e29808e71dca199f2d5f47f51360daeda23a8d24b747ce1c0</t>
+          <t>dc05f46018f671d923c8cc5092c9ae68d52498ea630593463d74e015787ed234</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -14043,7 +14807,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>4c8d9f6bbe98d1512f2b947bcbb304c485e39631d25f4f4b2d8c85f177b09bbf</t>
+          <t>e79ad66aa032a6374d1a831c706dc8703b8eecd34235271d481271751d50bd80</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -14077,7 +14841,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>008abe79eea6741fa9030c27a71c0e50d8702650313b6b2fbdc0d0f28341b07b</t>
+          <t>ad64473ae127fffe1404ae34767cab4bb81a1b56e65f4488ddf57f8eb49a5c63</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -14111,7 +14875,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>ad6f79268bd5323f45b576a49feeeb00132ebf51ceb5a6363b551582b5b5b695</t>
+          <t>a4bd3bb6ffef5fcb7b3d72420b7628d0a665f78f20c9da6fa8e5050e1ed153a5</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -14145,7 +14909,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>2322173a5acc464cda274b2196d499e047017ca6fbc6f5a7f21d9b38f8fc6029</t>
+          <t>3f391cb612a5c4d7577a3f1092587f75f0bd9619d637f95b889f0497c29dc573</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
@@ -14179,7 +14943,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>700df73ac171106a7daa05cf1cf1e961821550ced3c28f623bc56fd645c00b15</t>
+          <t>4c68afea5ce0a3a0486aeef94a16908ee4e274bfc17fc30542c6fa4f228efc10</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
@@ -14213,7 +14977,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>776b6cba8beb5f77f37c5aeb258fabbe3009a0d2a53ccc0d8a4753b4aaaaa250</t>
+          <t>18ae9b62c74038571f414eb59f6d44bd8cad790b1ee9aa3fdd3a38d3e40eb04a</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -14247,7 +15011,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>23d7b66b695fd7112748d15f930bf94be3938deba6761655cbbfa98389d0c4ab</t>
+          <t>0911a4961a25e6c03927b375611f5c1deb2c43cd55a0ab90bbe9af72bec46c04</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
@@ -14281,7 +15045,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>ea7e8873db1a5a56c5f8368aaa6cd7a8411706079a1743aef98757b0dbfc5a5e</t>
+          <t>a3b00b92ca010cace782ca085a1ca7c3d6544f474a78413c1d9861f7a1106acc</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
@@ -14315,7 +15079,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>98b8494a1f157a9192933ab82d26cacffa804384e0a6d27388cd3dee4b6db6ad</t>
+          <t>af0db871a5acb607e80792c4fedf36f03e4a734ba4d501282d4b228ff80baf98</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -14349,7 +15113,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>7864c7b0da953b0c8b3512533ea9c8ed4739abe92d0704aefe74aada48ae3a94</t>
+          <t>9ce150179196f03f1b2f92e53907025095fb12e3e774e01d570512ec600cb09a</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
@@ -14383,7 +15147,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>885d28a07e6dce54627ecfde7cdcfc4335c117b25a3a3825c9b4812a55b070ff</t>
+          <t>d46c4e7e9e83fa444a510bccc7b0ec3eb99ea6b77df0a928baaab7db91570c72</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
@@ -14417,7 +15181,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>3ed4c709b402b8f66b7761ee94036497add1b0584e2f773a3c435033dd42e45c</t>
+          <t>4c3740aff430fc03aec17021d27d34c0978a0a43df85c61c715da7592aa25f28</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
@@ -14451,7 +15215,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>f14c4ad82fd4f042c0f016714d56571d2d4d88b72a4fcad8a7dd97e3d2460424</t>
+          <t>36b8120d56d74fb384a57e654f33265d92d99222709127891efe4154dbe56364</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
@@ -14485,7 +15249,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>1d63172f5c50d915eb384e8827e3f8e07b8de3eb382c0a6789913e7c3ffb60a2</t>
+          <t>6b9451d09288a20ec4c743c27b1cb4d013867d0fbac118f76e9088a7e5137fd3</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
@@ -14519,7 +15283,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>956878781937c0e23c8099caee75d5b2181e32e541f36bf33b351dfc58302ba1</t>
+          <t>807018947ecd914179d240e481b933b48b6f9c0e4957523066784f2582b5a607</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
@@ -14553,7 +15317,7 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>f44b8354622127c63e28b55a2dd0abbffebff6d72814f4fda17d46b176485f65</t>
+          <t>d5ec0653eec19770af2b53ac422ef45417f3ea2b8fe4a1c9674125af2bd93cba</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
@@ -14587,7 +15351,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>d49bf1273968e91e2d2b5a76a10e7f039e5b5aba782a7ed57d93be7a9ebf412d</t>
+          <t>d21ab18835abd31b75043274818e95a3bf4c72835233c8911b15b729742359c2</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
@@ -14621,7 +15385,7 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>d4061309c40a443a8ac924d11cc2581a84d018fac99ae51c92b19ee30637113a</t>
+          <t>46dad4c7b7a10c163a2ea56ee33b43048c124c4fb4a3081bca748ab9856fa9f2</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
@@ -14655,7 +15419,7 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>5e218abd231444cb20dac20c5a71d6059c595bd98745fada92e7b57d6a4d52a6</t>
+          <t>5b6b5051cfd90883781565e1660742bc693988647bd604e8e62a3fcca671afdd</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
@@ -14689,7 +15453,7 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>d5bdeb422c2c9da45ee0332ab4f3219245a63b24cc84c4d132e752d5e69d0b16</t>
+          <t>20ebd619f76daa7f27bf5c4ae3866781e6ca67f41bf72482e8087155556d2e12</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
@@ -14723,7 +15487,7 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>1fe1636f3db4b6d6e6c9b784a0444ba3b42d214693547d817717d8733647e3fc</t>
+          <t>a119c42edb9baf8f60ab954bb53244970b0bcd1c2e64d293ebcb6962a2a8f3bf</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
@@ -14757,7 +15521,7 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>b48be9f95dd69e953ddb109a4798255f9f6e1bfb7be8976dff5b206902046865</t>
+          <t>06fc741a716df4985a3ec0726c08d880569420c9b0232bcefd04ebcc1b47e7e8</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
@@ -14791,7 +15555,7 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>2ec168861bc28a65b54b80bde27fbcf54cfdd1de472a5d5b6c9d6dbe476b6e14</t>
+          <t>f292dc2bfe344305fd9bce40a7998779de067fa8c56258e712e81222e870edff</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
@@ -14825,7 +15589,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>c1993dbe1de02998d5958fd91e936cc9da89e6409abe4ffcc098318a667764c1</t>
+          <t>c734795388881fd6771ed1001ef0ac850ad4dcd8ba01b8f124ac50308e60e9d5</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
@@ -14859,7 +15623,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>c70d647866eb59904c9e631b268d3ba3cf4d79f3fcf25302f507dbd273efdc74</t>
+          <t>f9f854081ca48cd022dd3e3df0ba0b39f2654a18d5a11df078b6ad21557fc063</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
@@ -14893,7 +15657,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>eada7b06041b7d6d9a216604dcaf54158112c83a2e78654c2e6d36cfaf0c5a93</t>
+          <t>c2e639a976e3441b816384c88356487fb94286182add6947df5eb470b4231d54</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
@@ -14927,7 +15691,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>7d4a9fadd4b1f2319eb296344b408d7589d1ae9f448ff104edc743dd0caa5344</t>
+          <t>6ca88a5884ed569179f332e06f1e60d506e267ace55bdb4c0081694f4dc0b761</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
@@ -14961,7 +15725,7 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>3ba0cef1c43a5135221de0f1866d0ad8a72274383cf36ce94a3539a2281b883f</t>
+          <t>305b1202b1adabf3281ce378c6d10cf07ba2835d0234b05ff498998e9e5adfe9</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
@@ -14995,7 +15759,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>9206a3c8395617077d7d3903232ff7111b474cf0926eccc9379c99530dde1f1f</t>
+          <t>4c490913195c591b3d4c392ea4f5844cc9e900ec43424605c12c0973450ee968</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
@@ -15029,7 +15793,7 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>02c178fd7ab0d0a09f46beaa3d519d6c4361ece0c806d354db1c8f8470ca2a8d</t>
+          <t>09ab4c27e39e6856df52c72c1bd8673eeafabf652731514d528552af289ee12b</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
@@ -15063,7 +15827,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>7fb73c9f80278128b4cac1b659fac2e2584215d6b84489477730dd621699b7ea</t>
+          <t>fa04808589a9571cb0cb4906722e33d8dc8d26abc7e01cd858ddd0b032a9d936</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
@@ -15097,7 +15861,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>f8706743d4d426647d9a397f6d897431b78d04d13941d959898a01135a6fea6d</t>
+          <t>8e5e7b6f1b1086b56e7d3b1595c9498ea9810133b2d2ee8539bcfc4d475e163e</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
@@ -15131,7 +15895,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>edf3884b1ca16e7e147ebe6aa64a98660331ef2b669a6870a9acd0d970069eea</t>
+          <t>d30718e2c348e2c016dbd6f5187dfddc8709af779156ce5090fd5cd93d2a0597</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
@@ -15165,7 +15929,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>c8766a934e12de039c8ec65033995169133afba7e3b22d8d432eafe852c3726c</t>
+          <t>dafa66d85fc4bf4562f9bef6e608190172ea0a8cf694b247aa91fee159afdbba</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
@@ -15199,7 +15963,7 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>0f5b4b180edc4bc0e701c5632c8b944d1c7d9ab4009f8c9aae7e7ccded7f9296</t>
+          <t>f70d4813a04c77bad204d9b7aa462cf675c564aac27ca75ce130a8406c725749</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
@@ -15233,7 +15997,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>d66bbc7102a143594ba047196a4798242ae07893432c69930d543d43e95cc2ce</t>
+          <t>c2dc6f55baee693a95da88e96a4442a5d4f2d7386eaef6f78b49254662a5f847</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
@@ -15267,7 +16031,7 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>8b5fd966597926106481ef5248a7df97770d8db44ed23a17f99a8ab2d3e35801</t>
+          <t>f4dbc50f27c892c6099167a85f6c73fa72f678cb2949ca7ba0a5466ef1e9842c</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
@@ -15301,7 +16065,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>5fbcb1593bd49f2e2035809eca1117d724be8e3af455cc889d9e0b5fae6c889f</t>
+          <t>16974cdbf8fac1f973b94f965ed6b71115656a7defb02ad9318efe183296d2d8</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
@@ -15335,7 +16099,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>4bb3d19291067f8293264446053714217478361a2fe06936ee37b68edd920bf7</t>
+          <t>93e16cc61d7bd192dbb36792af9df3df75e984d5d2855dae5e0041e953febbfa</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
@@ -15369,7 +16133,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>3f5c259bae2cb8874238f578249e70e8a3529065a7d8b7d558cda750679e7433</t>
+          <t>9dedd7bd6345035f0e6b021bce40a7970f53c8f4e464b542dea35fec797d3151</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
@@ -15403,7 +16167,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>8f9a6f7993afb387a0f9e23896f4c3dab28204fb26296580b2a7366e5a9a7024</t>
+          <t>c231bee3bd84c73cef2bf51f15dd34ea6285ed17924bde48a42469a663415479</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
@@ -15437,7 +16201,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>c7bc6ca897184d6758bb065185e137b57e4de04c9a6e116afbf0956b3618bb8b</t>
+          <t>968827151c4e2f4fbdcc5731ca7fe8e3db271a90ead63c7a3a9784b2e7609c2f</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
@@ -15471,7 +16235,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>7ebab596438547d3c9a9ea5bd5aa2f2993d18bdbec090c0298a8b9b1e517da0d</t>
+          <t>86d0844dc3e3d80b7618a6d8d0e0e03f755fb956c1f8d637672dafd1f38662f0</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
@@ -15505,7 +16269,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>be3c47c60abbf0bd223dba71d2beeb5c701ead63a2524633750089656d55d6fb</t>
+          <t>1c2f69a531a5b97f2b5b52f2f4516a531545493e4d0fff40212155904690b9d6</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
@@ -15539,7 +16303,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>b882a146cc9e1c92ea13d4b3447442182121b027e40a464979b494f03956c6fa</t>
+          <t>2d5f5f309e98490b177149c2f409aea4b89a2486022e4ca5d25582e08bfb870f</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
@@ -15573,7 +16337,7 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>6222bf33b052e12e310668c755515cbbfadb96c7a5f264ed709df0f70ce7723a</t>
+          <t>a4127079f96a15f99dd05395e4bc11a7e67f9c738ad666c523a33f420c789fb3</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
@@ -15607,7 +16371,7 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>66365f69accd56b8f863deeff9dcaeb92a4c884da81e1d3cabb9bb58db500a07</t>
+          <t>d1fcf98d40bb0e290a1e0e8df9ebd68b745b2100d87e5e916f21692aaa7ab253</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
@@ -15641,7 +16405,7 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>9226830dee3a704dccc2a23b87303cd1c1a95c0cf0d21313113729097b05ba2c</t>
+          <t>c826314bbd6f575eedd37101861a93329fdb07b2ef96c41d5ef45c4695ea1a60</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
@@ -15675,7 +16439,7 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>1eda6767501fcf3816be82f384e4f7b454d151de0895e2771488c67e6a91ad7c</t>
+          <t>5a08f208e70a0150ccd7f730e93b3e0a872676cd327eb848aafd1c26cd824473</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
@@ -15709,7 +16473,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>8c1949f6a3c60d55581027a0ef2240c48430df515e2fa0a6628d5ca0434fa6e6</t>
+          <t>c10b55b687a2c2c0ba16f790cda54529fe8b8566562b0f8370faddfd10239f77</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
@@ -15743,7 +16507,7 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>6bec50af5661d8d752f84e3c02a753386f68efdcbbb3dee411d439804f987b7e</t>
+          <t>350f929f4e7ccc8f646e20786de5837ce937cfe4f72668c2ffc99bb1ec53e6fe</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
@@ -15777,7 +16541,7 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>0f04ec1106dc09660340b4f6135b98b0b1cef59ea21e5b9488e6edc88608b4f5</t>
+          <t>3f8d475c695ba8d4083632ef455a677b2c023baec112f9d019c230c2cc36fd10</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
@@ -15811,7 +16575,7 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>c169a4d55f8c5f3011031657d6bfd2b48bf82174a017cad5641b99509d92c909</t>
+          <t>e3a4f8a63b19aa158a7a258a339c3f8bde19fcc89c04892fa494c15fe14add56</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
@@ -15845,7 +16609,7 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>8fceb79af5fd5518c6cdde9d7492cd7afbf3226fd8bc4635b975483d74de39d6</t>
+          <t>cca8029af1540deca002bb354c64675b48abe0e83c7f876bb9962dcd4aeef585</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
@@ -15879,7 +16643,7 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>d293d321fc545073f85d2e34a75f3c7ea3e9a37dc25e92230643912c075e7c4e</t>
+          <t>160846dd934865d6cd4ff4ed75f71103c31510cd4d9d9ca596327a26157e89d3</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
@@ -15913,7 +16677,7 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>c9ede1ddcc76fd5d8201181130ae9b8d7d3bc25d994ad2ddab710fa08baa0aa6</t>
+          <t>b5483f31d251eb21521e3345c86c7f405055ebb1cc296a24db16ce3d2dbfad9a</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
@@ -15947,7 +16711,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>b7bf5e56283009b0b82f7c3cb5f69973b40c8b994297b1dc28cc9c191870d608</t>
+          <t>bddef390244fce851f1a35bea8088f38be07a5f6247303366f7eedf594f970d4</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
@@ -15981,7 +16745,7 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>92f9c57d2a052d8be81911264296a6bbe3c2543ae3aa19b0b5558bbc8ca60e07</t>
+          <t>4862159c80df6f6d380990b26fdbccf5b1801ee27b459a05b22e632531b48223</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
@@ -16015,7 +16779,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>e6c410f94c7c4960bf16c0f875adeb77cd1df55da188491c635297c353352cf4</t>
+          <t>9a914bff1dc8bfaa296bfa5589af643310329323d53192e80719c29ffcfe2f1f</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
@@ -16049,7 +16813,7 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>803a0fa8c8ffdbc4b518a30590bc4c13bc6dd2f464d3145b648d86732eb489fb</t>
+          <t>462d0cdfb3d2e65ac051550391ed23ec9c3bd246fa6fff41edbf0690bc29f2a0</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
@@ -16083,7 +16847,7 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>ec84bea4c3d4ce0e068be92ee5602e72e3bd95baf57a23bba0000fd86d1d3480</t>
+          <t>377b10558b2507126ac33c3c940440317433fd4d7dd357230180b396e723be09</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">

</xml_diff>